<commit_message>
Fix 52 failing tests: import flow, selectors, timeouts, search retry, modal checkboxes
- Fix T4000 import flow to handle multi-step assign fields page
- Add search retry with backoff for Swinging Cardinal seed (search index lag)
- Add Customize Form dialog handling for loan/consignment seed creation
- Add explicit timeouts to all seed tests (60-120s based on complexity)
- Fix globalSearch helper: remove ArrowDown that caused 404 navigation
- Fix transaction tests: use label selectors instead of card clicks
- Fix edition set tests: use direct URL navigation for reliable routing
- Fix modal checkbox interactions: use evaluate() for custom checkboxes
- Fix navigation: use navigateTo helper and direct URLs instead of fragile menu clicks
- Make T4317, T4321, T4357 self-sufficient (create data if missing)
- Add waitFor calls before element interactions across all tests
- Switch playwright config to headed mode
</commit_message>
<xml_diff>
--- a/Files/1.25.2024 (1).xlsx
+++ b/Files/1.25.2024 (1).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nick/QATest/Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CBD20B2-1A3E-6A42-848E-2D750AA9A554}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56B0F70A-3A39-3042-8F17-B5761506F0F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15020" yWindow="1620" windowWidth="25380" windowHeight="26840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15020" yWindow="820" windowWidth="25380" windowHeight="26840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1.25.2024" sheetId="1" r:id="rId1"/>

</xml_diff>